<commit_message>
Added drought level counts by time. Also trying to add summer averages.
</commit_message>
<xml_diff>
--- a/output/palmer_drought_trendlines/region/Decade.xlsx
+++ b/output/palmer_drought_trendlines/region/Decade.xlsx
@@ -55,27 +55,27 @@
     <t>West Region</t>
   </si>
   <si>
+    <t>Great Basin</t>
+  </si>
+  <si>
+    <t>California River Basin</t>
+  </si>
+  <si>
     <t>US Rockies and Westward</t>
   </si>
   <si>
-    <t>Great Basin</t>
+    <t>Rio Grande River Basin</t>
   </si>
   <si>
     <t>NWS Western Region</t>
   </si>
   <si>
-    <t>California River Basin</t>
-  </si>
-  <si>
-    <t>Rio Grande River Basin</t>
+    <t>Spring Wheat Belt (area weighted)</t>
   </si>
   <si>
     <t>West North Central Region</t>
   </si>
   <si>
-    <t>Spring Wheat Belt (area weighted)</t>
-  </si>
-  <si>
     <t>Cotton Belt (area weighted)</t>
   </si>
   <si>
@@ -91,57 +91,57 @@
     <t>Northwest Region</t>
   </si>
   <si>
+    <t>Cotton Belt (productivity weighted)</t>
+  </si>
+  <si>
+    <t>Southeast Region</t>
+  </si>
+  <si>
     <t>Contiguous 48 States</t>
   </si>
   <si>
-    <t>Cotton Belt (productivity weighted)</t>
+    <t>South Atlantic-Gulf Basin</t>
   </si>
   <si>
     <t>Primary Hard Red Winter Wheat Belt (area weighted)</t>
   </si>
   <si>
-    <t>Southeast Region</t>
-  </si>
-  <si>
-    <t>South Atlantic-Gulf Basin</t>
+    <t>Souris-Red-Rainy Basin</t>
+  </si>
+  <si>
+    <t>NWS Southern Region</t>
+  </si>
+  <si>
+    <t>Spring Wheat Belt (productivity weighted)</t>
+  </si>
+  <si>
+    <t>NWS Eastern Region</t>
   </si>
   <si>
     <t>Southern Plains and Gulf Coast</t>
   </si>
   <si>
-    <t>NWS Southern Region</t>
-  </si>
-  <si>
-    <t>Souris-Red-Rainy Basin</t>
+    <t>Arkansas-White-Red Basin</t>
+  </si>
+  <si>
+    <t>Mid-Atlantic Basin</t>
   </si>
   <si>
     <t>Winter Wheat Belt (productivity weighted)</t>
   </si>
   <si>
-    <t>Spring Wheat Belt (productivity weighted)</t>
-  </si>
-  <si>
-    <t>Arkansas-White-Red Basin</t>
-  </si>
-  <si>
     <t>Winter Wheat Belt (area weighted)</t>
   </si>
   <si>
-    <t>NWS Eastern Region</t>
-  </si>
-  <si>
     <t>South Region</t>
   </si>
   <si>
-    <t>Mid-Atlantic Basin</t>
+    <t>Northeast Region</t>
   </si>
   <si>
     <t>Texas Gulf Coast River Basin</t>
   </si>
   <si>
-    <t>Northeast Region</t>
-  </si>
-  <si>
     <t>NWS Central Region</t>
   </si>
   <si>
@@ -154,37 +154,37 @@
     <t>Lower Mississippi River Basin</t>
   </si>
   <si>
+    <t>Tennessee River Basin</t>
+  </si>
+  <si>
+    <t>Soybean Belt (area weighted)</t>
+  </si>
+  <si>
     <t>Central Region</t>
   </si>
   <si>
+    <t>Ohio River Basin</t>
+  </si>
+  <si>
+    <t>Soybean Belt (productivity weighted)</t>
+  </si>
+  <si>
+    <t>East North Central Region</t>
+  </si>
+  <si>
     <t>Upper Mississippi River Basin</t>
   </si>
   <si>
-    <t>Ohio River Basin</t>
-  </si>
-  <si>
-    <t>East North Central Region</t>
-  </si>
-  <si>
-    <t>Tennessee River Basin</t>
-  </si>
-  <si>
-    <t>Soybean Belt (area weighted)</t>
-  </si>
-  <si>
-    <t>Soybean Belt (productivity weighted)</t>
-  </si>
-  <si>
     <t>Corn Belt (productivity weighted)</t>
   </si>
   <si>
+    <t>Primary Corn and Soybean Belt (area weighted)</t>
+  </si>
+  <si>
+    <t>Great Lakes Basin</t>
+  </si>
+  <si>
     <t>Corn Belt (area weighted)</t>
-  </si>
-  <si>
-    <t>Primary Corn and Soybean Belt (area weighted)</t>
-  </si>
-  <si>
-    <t>Great Lakes Basin</t>
   </si>
 </sst>
 </file>
@@ -582,25 +582,25 @@
         <v>9</v>
       </c>
       <c r="C2">
-        <v>-0.02478768299876161</v>
+        <v>-0.04139514314228129</v>
       </c>
       <c r="D2">
-        <v>1.458038455015688</v>
+        <v>2.271755278555077</v>
       </c>
       <c r="E2">
-        <v>-0.3529080893967783</v>
+        <v>-0.337080597389853</v>
       </c>
       <c r="F2">
-        <v>3.319108528125953E-05</v>
+        <v>7.742542704136124E-05</v>
       </c>
       <c r="G2">
-        <v>0.005763944308765417</v>
+        <v>0.01014035399186529</v>
       </c>
       <c r="H2">
         <v>132</v>
       </c>
       <c r="I2">
-        <v>-1.764360334823322</v>
+        <v>-3.109613329941491</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -611,25 +611,25 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <v>-0.02044440052443106</v>
+        <v>-0.03617100626838608</v>
       </c>
       <c r="D3">
-        <v>1.101747943695413</v>
+        <v>1.800273721699314</v>
       </c>
       <c r="E3">
-        <v>-0.2980827221911801</v>
+        <v>-0.3017307461159452</v>
       </c>
       <c r="F3">
-        <v>0.0005177561907511441</v>
+        <v>0.0004381622399571161</v>
       </c>
       <c r="G3">
-        <v>0.005741958533273088</v>
+        <v>0.01002400764620268</v>
       </c>
       <c r="H3">
         <v>132</v>
       </c>
       <c r="I3">
-        <v>-1.556024124480625</v>
+        <v>-2.901957093190877</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -640,25 +640,25 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>-0.01951455021278222</v>
+        <v>-0.03531165293622686</v>
       </c>
       <c r="D4">
-        <v>0.9167510387518021</v>
+        <v>1.726928008140424</v>
       </c>
       <c r="E4">
-        <v>-0.3122883078257873</v>
+        <v>-0.3105972414292575</v>
       </c>
       <c r="F4">
-        <v>0.0002669759653352008</v>
+        <v>0.0002893863740246028</v>
       </c>
       <c r="G4">
-        <v>0.005206537238623441</v>
+        <v>0.009478069962919222</v>
       </c>
       <c r="H4">
         <v>132</v>
       </c>
       <c r="I4">
-        <v>-1.620140488909886</v>
+        <v>-2.863586873569068</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -669,228 +669,228 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>-0.01894192657592557</v>
+        <v>-0.03474710421436446</v>
       </c>
       <c r="D5">
-        <v>0.8961472907657091</v>
+        <v>1.683413720003393</v>
       </c>
       <c r="E5">
-        <v>-0.3096658859953009</v>
+        <v>-0.3127304884033399</v>
       </c>
       <c r="F5">
-        <v>0.0003024605831910301</v>
+        <v>0.00026138726828553</v>
       </c>
       <c r="G5">
-        <v>0.005101161033104343</v>
+        <v>0.009256100100688424</v>
       </c>
       <c r="H5">
         <v>132</v>
       </c>
       <c r="I5">
-        <v>-1.566303164104615</v>
+        <v>-2.833709827863988</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6">
-        <v>-0.01829530285706832</v>
+        <v>-0.03227526890136914</v>
       </c>
       <c r="D6">
-        <v>0.8987838548291367</v>
+        <v>1.569325192911049</v>
       </c>
       <c r="E6">
-        <v>-0.3029177374492464</v>
+        <v>-0.2636952356758397</v>
       </c>
       <c r="F6">
-        <v>0.0004148049453367112</v>
+        <v>0.002250044569678197</v>
       </c>
       <c r="G6">
-        <v>0.0050482835117979</v>
+        <v>0.01035489952601771</v>
       </c>
       <c r="H6">
         <v>132</v>
       </c>
       <c r="I6">
-        <v>-1.479605516589745</v>
+        <v>-2.626459764266939</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>-0.01810159300124959</v>
+        <v>-0.03139422604021944</v>
       </c>
       <c r="D7">
-        <v>0.9432106334266097</v>
+        <v>1.547124056643772</v>
       </c>
       <c r="E7">
-        <v>-0.2720204273088529</v>
+        <v>-0.2999561636476684</v>
       </c>
       <c r="F7">
-        <v>0.001603493395343981</v>
+        <v>0.0004753526501403797</v>
       </c>
       <c r="G7">
-        <v>0.005616299258412658</v>
+        <v>0.008756837409324552</v>
       </c>
       <c r="H7">
         <v>132</v>
       </c>
       <c r="I7">
-        <v>-1.409996456735837</v>
+        <v>-2.534125328584754</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8">
-        <v>-0.01679288854535612</v>
+        <v>-0.02858190451963031</v>
       </c>
       <c r="D8">
-        <v>0.9143198931569583</v>
+        <v>1.321528194691767</v>
       </c>
       <c r="E8">
-        <v>-0.2908130994334771</v>
+        <v>-0.261836986551212</v>
       </c>
       <c r="F8">
-        <v>0.0007174341831655274</v>
+        <v>0.002423288308762381</v>
       </c>
       <c r="G8">
-        <v>0.00484564728863534</v>
+        <v>0.00923987850449612</v>
       </c>
       <c r="H8">
         <v>132</v>
       </c>
       <c r="I8">
-        <v>-1.268755617739338</v>
+        <v>-2.394119392860172</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
       </c>
       <c r="C9">
-        <v>-0.01534874636937726</v>
+        <v>-0.02856707042639376</v>
       </c>
       <c r="D9">
-        <v>0.7015130585940815</v>
+        <v>1.272948359196134</v>
       </c>
       <c r="E9">
-        <v>-0.2912880055189675</v>
+        <v>-0.2434649843393746</v>
       </c>
       <c r="F9">
-        <v>0.0007024912647493211</v>
+        <v>0.004907362549638044</v>
       </c>
       <c r="G9">
-        <v>0.004421046487809752</v>
+        <v>0.009981339263671994</v>
       </c>
       <c r="H9">
         <v>132</v>
       </c>
       <c r="I9">
-        <v>-1.293823969424962</v>
+        <v>-2.440770796235055</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
       </c>
       <c r="C10">
-        <v>-0.01524650873166519</v>
+        <v>-0.02628635109484768</v>
       </c>
       <c r="D10">
-        <v>0.5874373781056561</v>
+        <v>1.274122106334267</v>
       </c>
       <c r="E10">
-        <v>-0.2321499449341137</v>
+        <v>-0.2457887378624516</v>
       </c>
       <c r="F10">
-        <v>0.007394654489928174</v>
+        <v>0.004500727095305147</v>
       </c>
       <c r="G10">
-        <v>0.005602735709361287</v>
+        <v>0.009092124112793688</v>
       </c>
       <c r="H10">
         <v>132</v>
       </c>
       <c r="I10">
-        <v>-1.394608757010818</v>
+        <v>-2.143103535995931</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
       <c r="C11">
-        <v>-0.01116752436489146</v>
+        <v>-0.02272196283323224</v>
       </c>
       <c r="D11">
-        <v>1.304781522937336</v>
+        <v>1.67842143644535</v>
       </c>
       <c r="E11">
-        <v>-0.1508934011015162</v>
+        <v>-0.1936126638574839</v>
       </c>
       <c r="F11">
-        <v>0.08415916999794891</v>
+        <v>0.02612324494640033</v>
       </c>
       <c r="G11">
-        <v>0.00641672818750152</v>
+        <v>0.01009819997947849</v>
       </c>
       <c r="H11">
         <v>132</v>
       </c>
       <c r="I11">
-        <v>-0.1469966444985529</v>
+        <v>-1.275433731874842</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
         <v>19</v>
       </c>
       <c r="C12">
-        <v>-0.01095198977228996</v>
+        <v>-0.02211913455831034</v>
       </c>
       <c r="D12">
-        <v>1.137715890782668</v>
+        <v>1.803972186890528</v>
       </c>
       <c r="E12">
-        <v>-0.1586227219078554</v>
+        <v>-0.1843308831938877</v>
       </c>
       <c r="F12">
-        <v>0.06927499262393431</v>
+        <v>0.034359819571199</v>
       </c>
       <c r="G12">
-        <v>0.005978914814840862</v>
+        <v>0.01034408039449808</v>
       </c>
       <c r="H12">
         <v>132</v>
       </c>
       <c r="I12">
-        <v>-0.2860427796150262</v>
+        <v>-1.071515305689816</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -901,25 +901,25 @@
         <v>20</v>
       </c>
       <c r="C13">
-        <v>-0.009890396286491432</v>
+        <v>-0.02164318598386267</v>
       </c>
       <c r="D13">
-        <v>0.5353949800729249</v>
+        <v>1.094384974137201</v>
       </c>
       <c r="E13">
-        <v>-0.1575958128257301</v>
+        <v>-0.186838774898026</v>
       </c>
       <c r="F13">
-        <v>0.0711198005695922</v>
+        <v>0.03194290485987202</v>
       </c>
       <c r="G13">
-        <v>0.005435457127196858</v>
+        <v>0.009980830917127408</v>
       </c>
       <c r="H13">
         <v>132</v>
       </c>
       <c r="I13">
-        <v>-0.7503565371709614</v>
+        <v>-1.719229203764946</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -930,25 +930,25 @@
         <v>21</v>
       </c>
       <c r="C14">
-        <v>-0.008949755395965016</v>
+        <v>-0.01892619480917624</v>
       </c>
       <c r="D14">
-        <v>1.147991435597389</v>
+        <v>1.635104723140847</v>
       </c>
       <c r="E14">
-        <v>-0.1181741888420323</v>
+        <v>-0.1554692001344543</v>
       </c>
       <c r="F14">
-        <v>0.1771640832204904</v>
+        <v>0.0750667777709185</v>
       </c>
       <c r="G14">
-        <v>0.006595731903318887</v>
+        <v>0.01054712756796859</v>
       </c>
       <c r="H14">
         <v>132</v>
       </c>
       <c r="I14">
-        <v>-0.01547676587806346</v>
+        <v>-0.8253006020520652</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -959,25 +959,25 @@
         <v>22</v>
       </c>
       <c r="C15">
-        <v>-0.006614652993068159</v>
+        <v>-0.018739319935555</v>
       </c>
       <c r="D15">
-        <v>0.9745720342576107</v>
+        <v>1.636309166454677</v>
       </c>
       <c r="E15">
-        <v>-0.09407565319245134</v>
+        <v>-0.1561498088603786</v>
       </c>
       <c r="F15">
-        <v>0.2832942757157758</v>
+        <v>0.07378478231576593</v>
       </c>
       <c r="G15">
-        <v>0.006139426294298623</v>
+        <v>0.01039633882955093</v>
       </c>
       <c r="H15">
         <v>132</v>
       </c>
       <c r="I15">
-        <v>0.11466714515875</v>
+        <v>-0.7998024251674727</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -988,25 +988,25 @@
         <v>23</v>
       </c>
       <c r="C16">
-        <v>-0.006411548292291109</v>
+        <v>-0.01715543771076716</v>
       </c>
       <c r="D16">
-        <v>0.1181444076994829</v>
+        <v>0.6193979479352166</v>
       </c>
       <c r="E16">
-        <v>-0.1466024589592265</v>
+        <v>-0.1781867399206297</v>
       </c>
       <c r="F16">
-        <v>0.09346632594455273</v>
+        <v>0.04094099022317375</v>
       </c>
       <c r="G16">
-        <v>0.00379430392267737</v>
+        <v>0.008308992797725694</v>
       </c>
       <c r="H16">
         <v>132</v>
       </c>
       <c r="I16">
-        <v>-0.7153568702983614</v>
+        <v>-1.610808954464514</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1017,199 +1017,199 @@
         <v>24</v>
       </c>
       <c r="C17">
-        <v>-0.005669839390661068</v>
+        <v>-0.01631631671982728</v>
       </c>
       <c r="D17">
-        <v>0.08206270669040983</v>
+        <v>0.555846858305775</v>
       </c>
       <c r="E17">
-        <v>-0.1308914971114055</v>
+        <v>-0.1692474081945817</v>
       </c>
       <c r="F17">
-        <v>0.1346616307205111</v>
+        <v>0.05237607573357037</v>
       </c>
       <c r="G17">
-        <v>0.003766475218566067</v>
+        <v>0.008333308973065154</v>
       </c>
       <c r="H17">
         <v>132</v>
       </c>
       <c r="I17">
-        <v>-0.655016414095529</v>
+        <v>-1.565274315271772</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
       </c>
       <c r="C18">
-        <v>-0.003960743148990416</v>
+        <v>-0.01594229171151074</v>
       </c>
       <c r="D18">
-        <v>0.4212083439328416</v>
+        <v>0.7082123293479186</v>
       </c>
       <c r="E18">
-        <v>-0.06392775414549851</v>
+        <v>-0.146821513765262</v>
       </c>
       <c r="F18">
-        <v>0.4664706063680815</v>
+        <v>0.09297220942991884</v>
       </c>
       <c r="G18">
-        <v>0.005422833990936239</v>
+        <v>0.009420137491761094</v>
       </c>
       <c r="H18">
         <v>132</v>
       </c>
       <c r="I18">
-        <v>-0.09368826543591247</v>
+        <v>-1.364285593148478</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
       </c>
       <c r="C19">
-        <v>-0.003319903639987591</v>
+        <v>-0.01426078964705269</v>
       </c>
       <c r="D19">
-        <v>0.0636818451623847</v>
+        <v>0.5930920037310273</v>
       </c>
       <c r="E19">
-        <v>-0.06084932027355858</v>
+        <v>-0.1476641176195292</v>
       </c>
       <c r="F19">
-        <v>0.4882475739633817</v>
+        <v>0.09109085780724646</v>
       </c>
       <c r="G19">
-        <v>0.004776310600385042</v>
+        <v>0.008377408844499806</v>
       </c>
       <c r="H19">
         <v>132</v>
       </c>
       <c r="I19">
-        <v>-0.3679056280360021</v>
+        <v>-1.260810650385823</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
       </c>
       <c r="C20">
-        <v>-0.002369780639101421</v>
+        <v>-0.01415194933108951</v>
       </c>
       <c r="D20">
-        <v>0.4023165861104043</v>
+        <v>0.8501273636903252</v>
       </c>
       <c r="E20">
-        <v>-0.03762521576655055</v>
+        <v>-0.1311743862188633</v>
       </c>
       <c r="F20">
-        <v>0.6684174126887185</v>
+        <v>0.1338137762503171</v>
       </c>
       <c r="G20">
-        <v>0.005520136894112678</v>
+        <v>0.009380514028818012</v>
       </c>
       <c r="H20">
         <v>132</v>
       </c>
       <c r="I20">
-        <v>0.09424510302721961</v>
+        <v>-0.9896260493513106</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="B21" t="s">
         <v>28</v>
       </c>
       <c r="C21">
-        <v>-0.001799980664633425</v>
+        <v>-0.01400653973347945</v>
       </c>
       <c r="D21">
-        <v>-0.01782035953531749</v>
+        <v>0.584143644534894</v>
       </c>
       <c r="E21">
-        <v>-0.04103600465739753</v>
+        <v>-0.1454239875277568</v>
       </c>
       <c r="F21">
-        <v>0.6403707860430112</v>
+        <v>0.09616040879051212</v>
       </c>
       <c r="G21">
-        <v>0.003843838383718956</v>
+        <v>0.008357600711645338</v>
       </c>
       <c r="H21">
         <v>132</v>
       </c>
       <c r="I21">
-        <v>-0.2518178459376628</v>
+        <v>-1.236706520817434</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
       </c>
       <c r="C22">
-        <v>-0.001406986496925444</v>
+        <v>-0.01346308174992989</v>
       </c>
       <c r="D22">
-        <v>-0.03932922072415843</v>
+        <v>0.9373998134486564</v>
       </c>
       <c r="E22">
-        <v>-0.03242226645699833</v>
+        <v>-0.1202424119937283</v>
       </c>
       <c r="F22">
-        <v>0.7120848066147334</v>
+        <v>0.1696501584111955</v>
       </c>
       <c r="G22">
-        <v>0.003804052453226372</v>
+        <v>0.009748833283525426</v>
       </c>
       <c r="H22">
         <v>132</v>
       </c>
       <c r="I22">
-        <v>-0.2222374653244661</v>
+        <v>-0.812800814042229</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23">
-        <v>-0.0002062013412687536</v>
+        <v>-0.01171556920989636</v>
       </c>
       <c r="D23">
-        <v>-0.1786746798948528</v>
+        <v>1.330146018824727</v>
       </c>
       <c r="E23">
-        <v>-0.003233288686235161</v>
+        <v>-0.1101117420293871</v>
       </c>
       <c r="F23">
-        <v>0.9706489124472601</v>
+        <v>0.2087967948026354</v>
       </c>
       <c r="G23">
-        <v>0.005593363667129958</v>
+        <v>0.009274898608498446</v>
       </c>
       <c r="H23">
         <v>132</v>
       </c>
       <c r="I23">
-        <v>-0.2054808542597908</v>
+        <v>-0.1928779784617998</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1220,112 +1220,112 @@
         <v>31</v>
       </c>
       <c r="C24">
-        <v>0.0006983386028031153</v>
+        <v>-0.01112215590735052</v>
       </c>
       <c r="D24">
-        <v>-0.1702617654540829</v>
+        <v>0.3884139743915886</v>
       </c>
       <c r="E24">
-        <v>0.01143762057608374</v>
+        <v>-0.1008370005386396</v>
       </c>
       <c r="F24">
-        <v>0.8964377394449357</v>
+        <v>0.2499606696417918</v>
       </c>
       <c r="G24">
-        <v>0.005354640015445584</v>
+        <v>0.009624498440692549</v>
       </c>
       <c r="H24">
         <v>132</v>
       </c>
       <c r="I24">
-        <v>-0.07947774708967796</v>
+        <v>-1.057466293563979</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="B25" t="s">
         <v>32</v>
       </c>
       <c r="C25">
-        <v>0.001185606892895114</v>
+        <v>-0.01109717237735555</v>
       </c>
       <c r="D25">
-        <v>0.6546367760535912</v>
+        <v>1.208154328839143</v>
       </c>
       <c r="E25">
-        <v>0.02035706505038529</v>
+        <v>-0.09765996738072406</v>
       </c>
       <c r="F25">
-        <v>0.8167831879371057</v>
+        <v>0.26527014925123</v>
       </c>
       <c r="G25">
-        <v>0.005106976604492069</v>
+        <v>0.009918433972281317</v>
       </c>
       <c r="H25">
         <v>132</v>
       </c>
       <c r="I25">
-        <v>0.808765672129956</v>
+        <v>-0.2344780802170787</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>33</v>
       </c>
       <c r="C26">
-        <v>0.001493376169323764</v>
+        <v>-0.01060097319792054</v>
       </c>
       <c r="D26">
-        <v>0.2670811922326805</v>
+        <v>0.6505389637920803</v>
       </c>
       <c r="E26">
-        <v>0.02376782756889485</v>
+        <v>-0.1127092630420259</v>
       </c>
       <c r="F26">
-        <v>0.7867659820559455</v>
+        <v>0.1981923509912407</v>
       </c>
       <c r="G26">
-        <v>0.00550915953979035</v>
+        <v>0.008196685573309574</v>
       </c>
       <c r="H26">
         <v>132</v>
       </c>
       <c r="I26">
-        <v>0.4612200942447699</v>
+        <v>-0.7275875519375904</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
         <v>34</v>
       </c>
       <c r="C27">
-        <v>0.001509927755615878</v>
+        <v>-0.01059903202029888</v>
       </c>
       <c r="D27">
-        <v>0.5298553803103534</v>
+        <v>0.2516229966929538</v>
       </c>
       <c r="E27">
-        <v>0.02387819447512102</v>
+        <v>-0.09375859925324567</v>
       </c>
       <c r="F27">
-        <v>0.7857996278159466</v>
+        <v>0.2849271762118099</v>
       </c>
       <c r="G27">
-        <v>0.005544458811457004</v>
+        <v>0.009871112628624003</v>
       </c>
       <c r="H27">
         <v>132</v>
       </c>
       <c r="I27">
-        <v>0.7261459885404176</v>
+        <v>-1.1262511659459</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1336,199 +1336,199 @@
         <v>35</v>
       </c>
       <c r="C28">
-        <v>0.001931864171612329</v>
+        <v>-0.009172651312056046</v>
       </c>
       <c r="D28">
-        <v>0.06954553548715331</v>
+        <v>0.6411650979394559</v>
       </c>
       <c r="E28">
-        <v>0.03265966581104477</v>
+        <v>-0.08459230737400661</v>
       </c>
       <c r="F28">
-        <v>0.7100705814200485</v>
+        <v>0.3348566203071313</v>
       </c>
       <c r="G28">
-        <v>0.00518515127038271</v>
+        <v>0.00947617071676689</v>
       </c>
       <c r="H28">
         <v>132</v>
       </c>
       <c r="I28">
-        <v>0.3206878777967561</v>
+        <v>-0.5512795726278301</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
         <v>36</v>
       </c>
       <c r="C29">
-        <v>0.002250105249621915</v>
+        <v>-0.008541154139678694</v>
       </c>
       <c r="D29">
-        <v>0.2722035529551428</v>
+        <v>0.4129049436106169</v>
       </c>
       <c r="E29">
-        <v>0.03523167147345033</v>
+        <v>-0.09128456698547943</v>
       </c>
       <c r="F29">
-        <v>0.6883791270795585</v>
+        <v>0.2978848877178756</v>
       </c>
       <c r="G29">
-        <v>0.005597939534734769</v>
+        <v>0.008172039971839774</v>
       </c>
       <c r="H29">
         <v>132</v>
       </c>
       <c r="I29">
-        <v>0.5647172354059917</v>
+        <v>-0.6974450945476134</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B30" t="s">
         <v>37</v>
       </c>
       <c r="C30">
-        <v>0.002679692973015285</v>
+        <v>-0.0076459933859069</v>
       </c>
       <c r="D30">
-        <v>-0.04342898329517522</v>
+        <v>0.616186381751887</v>
       </c>
       <c r="E30">
-        <v>0.06561371171402633</v>
+        <v>-0.07027766620948486</v>
       </c>
       <c r="F30">
-        <v>0.4547737663792559</v>
+        <v>0.423282178048217</v>
       </c>
       <c r="G30">
-        <v>0.00357422496181193</v>
+        <v>0.009518527615568142</v>
       </c>
       <c r="H30">
         <v>132</v>
       </c>
       <c r="I30">
-        <v>0.3049311031968118</v>
+        <v>-0.37779275841601</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
       </c>
       <c r="C31">
-        <v>0.00365053356293499</v>
+        <v>-0.007337770124389307</v>
       </c>
       <c r="D31">
-        <v>-0.302060459594675</v>
+        <v>0.6308735690663954</v>
       </c>
       <c r="E31">
-        <v>0.05993743682714006</v>
+        <v>-0.06669628438731372</v>
       </c>
       <c r="F31">
-        <v>0.4948007480586825</v>
+        <v>0.4473500435800749</v>
       </c>
       <c r="G31">
-        <v>0.005332182404911103</v>
+        <v>0.009627702774319669</v>
       </c>
       <c r="H31">
         <v>132</v>
       </c>
       <c r="I31">
-        <v>0.1725089035868738</v>
+        <v>-0.3230365471042145</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
       </c>
       <c r="C32">
-        <v>0.004152277799365057</v>
+        <v>-0.006346183198638048</v>
       </c>
       <c r="D32">
-        <v>-0.2406198168404988</v>
+        <v>0.1371610277283136</v>
       </c>
       <c r="E32">
-        <v>0.101878832184979</v>
+        <v>-0.0570861314870384</v>
       </c>
       <c r="F32">
-        <v>0.2450758374194758</v>
+        <v>0.5155875207511315</v>
       </c>
       <c r="G32">
-        <v>0.003556027847860649</v>
+        <v>0.009734228006570016</v>
       </c>
       <c r="H32">
         <v>132</v>
       </c>
       <c r="I32">
-        <v>0.2991762970769586</v>
+        <v>-0.6878427880946327</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="B33" t="s">
         <v>40</v>
       </c>
       <c r="C33">
-        <v>0.005155734310631287</v>
+        <v>-0.005375110397954461</v>
       </c>
       <c r="D33">
-        <v>-0.516663190027983</v>
+        <v>0.2093223098448234</v>
       </c>
       <c r="E33">
-        <v>0.08483779714803022</v>
+        <v>-0.05791762994862039</v>
       </c>
       <c r="F33">
-        <v>0.3334508410603355</v>
+        <v>0.5094797590737756</v>
       </c>
       <c r="G33">
-        <v>0.005310811792811101</v>
+        <v>0.008125971526367329</v>
       </c>
       <c r="H33">
         <v>132</v>
       </c>
       <c r="I33">
-        <v>0.1535822703540842</v>
+        <v>-0.4894420418892564</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B34" t="s">
         <v>41</v>
       </c>
       <c r="C34">
-        <v>0.00693656415660995</v>
+        <v>-0.004730454180772167</v>
       </c>
       <c r="D34">
-        <v>-0.4058719155431191</v>
+        <v>-0.1428616976172304</v>
       </c>
       <c r="E34">
-        <v>0.168783287747052</v>
+        <v>-0.04243563364357255</v>
       </c>
       <c r="F34">
-        <v>0.05303548410614849</v>
+        <v>0.6290042408869247</v>
       </c>
       <c r="G34">
-        <v>0.003552772665244827</v>
+        <v>0.009768077241313478</v>
       </c>
       <c r="H34">
         <v>132</v>
       </c>
       <c r="I34">
-        <v>0.4958814248161744</v>
+        <v>-0.7578207411176121</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1539,25 +1539,25 @@
         <v>42</v>
       </c>
       <c r="C35">
-        <v>0.007250369701527172</v>
+        <v>-0.004600700545956208</v>
       </c>
       <c r="D35">
-        <v>-0.000790087339947676</v>
+        <v>0.5269098617824135</v>
       </c>
       <c r="E35">
-        <v>0.1270088920074764</v>
+        <v>-0.04453821376355798</v>
       </c>
       <c r="F35">
-        <v>0.1467169094357887</v>
+        <v>0.6120917194266923</v>
       </c>
       <c r="G35">
-        <v>0.004966185413305793</v>
+        <v>0.009050828224642864</v>
       </c>
       <c r="H35">
         <v>132</v>
       </c>
       <c r="I35">
-        <v>0.9417579738585846</v>
+        <v>-0.07118120919189352</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1568,25 +1568,25 @@
         <v>43</v>
       </c>
       <c r="C36">
-        <v>0.007723286909817059</v>
+        <v>-0.003576915901871386</v>
       </c>
       <c r="D36">
-        <v>0.09607182226744659</v>
+        <v>0.5506939709997458</v>
       </c>
       <c r="E36">
-        <v>0.1259311390359526</v>
+        <v>-0.03426917256478689</v>
       </c>
       <c r="F36">
-        <v>0.1502037786609078</v>
+        <v>0.6964680347123431</v>
       </c>
       <c r="G36">
-        <v>0.005336126300751242</v>
+        <v>0.009149097850015055</v>
       </c>
       <c r="H36">
         <v>132</v>
       </c>
       <c r="I36">
-        <v>1.100099120543664</v>
+        <v>0.0856949037564656</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1597,25 +1597,25 @@
         <v>44</v>
       </c>
       <c r="C37">
-        <v>0.008147467532891094</v>
+        <v>-0.002987117520823957</v>
       </c>
       <c r="D37">
-        <v>-0.4861068854405159</v>
+        <v>0.06932671924022732</v>
       </c>
       <c r="E37">
-        <v>0.2040985046768775</v>
+        <v>-0.03260421133510322</v>
       </c>
       <c r="F37">
-        <v>0.01890618589475416</v>
+        <v>0.7105409087704093</v>
       </c>
       <c r="G37">
-        <v>0.003427455369349632</v>
+        <v>0.008031117422189357</v>
       </c>
       <c r="H37">
         <v>132</v>
       </c>
       <c r="I37">
-        <v>0.5730638938353263</v>
+        <v>-0.3189985584668871</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1626,228 +1626,228 @@
         <v>45</v>
       </c>
       <c r="C38">
-        <v>0.008721343542406888</v>
+        <v>-0.002830833153957043</v>
       </c>
       <c r="D38">
-        <v>-0.6989144831679812</v>
+        <v>-0.1248493173916729</v>
       </c>
       <c r="E38">
-        <v>0.2023224645321595</v>
+        <v>-0.02947643138667949</v>
       </c>
       <c r="F38">
-        <v>0.01999115421664287</v>
+        <v>0.7372401883157859</v>
       </c>
       <c r="G38">
-        <v>0.003702471915342312</v>
+        <v>0.008419357306524928</v>
       </c>
       <c r="H38">
         <v>132</v>
       </c>
       <c r="I38">
-        <v>0.4348601773449141</v>
+        <v>-0.4928576274060885</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="B39" t="s">
         <v>46</v>
       </c>
       <c r="C39">
-        <v>0.01076197376353826</v>
+        <v>-0.002061627171268483</v>
       </c>
       <c r="D39">
-        <v>-0.5232071143898926</v>
+        <v>0.1927533282455694</v>
       </c>
       <c r="E39">
-        <v>0.2154848739107032</v>
+        <v>-0.02174111917405279</v>
       </c>
       <c r="F39">
-        <v>0.01308639360948242</v>
+        <v>0.8045677845257424</v>
       </c>
       <c r="G39">
-        <v>0.004277390523149407</v>
+        <v>0.008314839910834574</v>
       </c>
       <c r="H39">
         <v>132</v>
       </c>
       <c r="I39">
-        <v>0.8758494748700807</v>
+        <v>-0.07525820401933342</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B40" t="s">
         <v>47</v>
       </c>
       <c r="C40">
-        <v>0.01077612240638189</v>
+        <v>0.0007342086896398799</v>
       </c>
       <c r="D40">
-        <v>-0.1926075214110068</v>
+        <v>0.1826644619689645</v>
       </c>
       <c r="E40">
-        <v>0.2080834549712171</v>
+        <v>0.007316953672887244</v>
       </c>
       <c r="F40">
-        <v>0.01665543576290289</v>
+        <v>0.9336392840289326</v>
       </c>
       <c r="G40">
-        <v>0.004442643514916126</v>
+        <v>0.008800470933456725</v>
       </c>
       <c r="H40">
         <v>132</v>
       </c>
       <c r="I40">
-        <v>1.208288391418639</v>
+        <v>0.2781115916221488</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="B41" t="s">
         <v>48</v>
       </c>
       <c r="C41">
-        <v>0.01136313304689037</v>
+        <v>0.001042752871651372</v>
       </c>
       <c r="D41">
-        <v>-0.5664621809548043</v>
+        <v>-0.1316089205460867</v>
       </c>
       <c r="E41">
-        <v>0.241464879259793</v>
+        <v>0.01081327883063006</v>
       </c>
       <c r="F41">
-        <v>0.005283336238007865</v>
+        <v>0.9020618974316522</v>
       </c>
       <c r="G41">
-        <v>0.004005230450234806</v>
+        <v>0.008457206300937121</v>
       </c>
       <c r="H41">
         <v>132</v>
       </c>
       <c r="I41">
-        <v>0.9107451151409436</v>
+        <v>0.003948952768591613</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="B42" t="s">
         <v>49</v>
       </c>
       <c r="C42">
-        <v>0.01170769487021078</v>
+        <v>0.001146141452882744</v>
       </c>
       <c r="D42">
-        <v>-0.3561569151191389</v>
+        <v>-0.1218653438480456</v>
       </c>
       <c r="E42">
-        <v>0.2358577728017027</v>
+        <v>0.01221387317811288</v>
       </c>
       <c r="F42">
-        <v>0.00647808232138066</v>
+        <v>0.8894523451003896</v>
       </c>
       <c r="G42">
-        <v>0.004230784186898347</v>
+        <v>0.008229638177953332</v>
       </c>
       <c r="H42">
         <v>132</v>
       </c>
       <c r="I42">
-        <v>1.165843418008262</v>
+        <v>0.02713304502671107</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B43" t="s">
         <v>50</v>
       </c>
       <c r="C43">
-        <v>0.01177909744372477</v>
+        <v>0.001529041347866078</v>
       </c>
       <c r="D43">
-        <v>-0.6465285762740609</v>
+        <v>0.06554583227338232</v>
       </c>
       <c r="E43">
-        <v>0.2517657073940855</v>
+        <v>0.01529137428838767</v>
       </c>
       <c r="F43">
-        <v>0.0035898913361145</v>
+        <v>0.8618468272478064</v>
       </c>
       <c r="G43">
-        <v>0.003971221328505517</v>
+        <v>0.008769003716384246</v>
       </c>
       <c r="H43">
         <v>132</v>
       </c>
       <c r="I43">
-        <v>0.8847540914101586</v>
+        <v>0.2643212074959725</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="B44" t="s">
         <v>51</v>
       </c>
       <c r="C44">
-        <v>0.01180151072111134</v>
+        <v>0.001534016920076445</v>
       </c>
       <c r="D44">
-        <v>-0.2868116255405753</v>
+        <v>0.06678317646061233</v>
       </c>
       <c r="E44">
-        <v>0.2126680300255295</v>
+        <v>0.01608230861241003</v>
       </c>
       <c r="F44">
-        <v>0.01435703269031585</v>
+        <v>0.8547775491175317</v>
       </c>
       <c r="G44">
-        <v>0.004755690996415141</v>
+        <v>0.008364768220067193</v>
       </c>
       <c r="H44">
         <v>132</v>
       </c>
       <c r="I44">
-        <v>1.247384768203898</v>
+        <v>0.2662053760705502</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="B45" t="s">
         <v>52</v>
       </c>
       <c r="C45">
-        <v>0.01211187154234726</v>
+        <v>0.001811862317280784</v>
       </c>
       <c r="D45">
-        <v>-0.3559749003646236</v>
+        <v>0.1399899940642756</v>
       </c>
       <c r="E45">
-        <v>0.2204020415661003</v>
+        <v>0.01860305976716366</v>
       </c>
       <c r="F45">
-        <v>0.01110267502397392</v>
+        <v>0.8323267761670338</v>
       </c>
       <c r="G45">
-        <v>0.004701222177393609</v>
+        <v>0.008540709952715978</v>
       </c>
       <c r="H45">
         <v>132</v>
       </c>
       <c r="I45">
-        <v>1.21856840014052</v>
+        <v>0.3755320953107775</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -1858,112 +1858,112 @@
         <v>53</v>
       </c>
       <c r="C46">
-        <v>0.01211502031844185</v>
+        <v>0.001958350781754498</v>
       </c>
       <c r="D46">
-        <v>-0.2760681336385999</v>
+        <v>0.1050209446281692</v>
       </c>
       <c r="E46">
-        <v>0.207439182670127</v>
+        <v>0.01928054194778564</v>
       </c>
       <c r="F46">
-        <v>0.01700275507307683</v>
+        <v>0.8263150516329765</v>
       </c>
       <c r="G46">
-        <v>0.005010840853051454</v>
+        <v>0.008906741238857836</v>
       </c>
       <c r="H46">
         <v>132</v>
       </c>
       <c r="I46">
-        <v>1.29888450775884</v>
+        <v>0.3596065462562539</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B47" t="s">
         <v>54</v>
       </c>
       <c r="C47">
-        <v>0.01256710150275401</v>
+        <v>0.002319669425800183</v>
       </c>
       <c r="D47">
-        <v>-0.2211331298227768</v>
+        <v>0.005093530060205131</v>
       </c>
       <c r="E47">
-        <v>0.2137423230303633</v>
+        <v>0.02346323034333412</v>
       </c>
       <c r="F47">
-        <v>0.01386027885759906</v>
+        <v>0.7894346650380903</v>
       </c>
       <c r="G47">
-        <v>0.00503754129152343</v>
+        <v>0.008668561616183641</v>
       </c>
       <c r="H47">
         <v>132</v>
       </c>
       <c r="I47">
-        <v>1.412590065535245</v>
+        <v>0.3066505554142289</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B48" t="s">
         <v>55</v>
       </c>
       <c r="C48">
-        <v>0.01287925147437994</v>
+        <v>0.002615143272736762</v>
       </c>
       <c r="D48">
-        <v>-0.4108212074959724</v>
+        <v>-0.1466759942338675</v>
       </c>
       <c r="E48">
-        <v>0.2427300055616116</v>
+        <v>0.02931594946527999</v>
       </c>
       <c r="F48">
-        <v>0.005042647387199914</v>
+        <v>0.7386189008206709</v>
       </c>
       <c r="G48">
-        <v>0.004514495742944402</v>
+        <v>0.007820475224488361</v>
       </c>
       <c r="H48">
         <v>132</v>
       </c>
       <c r="I48">
-        <v>1.263481484173421</v>
+        <v>0.1932926312219115</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="B49" t="s">
         <v>56</v>
       </c>
       <c r="C49">
-        <v>0.01492694171342099</v>
+        <v>0.003144398567598771</v>
       </c>
       <c r="D49">
-        <v>-0.7292927160179772</v>
+        <v>0.06289612481980841</v>
       </c>
       <c r="E49">
-        <v>0.3392230654971448</v>
+        <v>0.03126881341251011</v>
       </c>
       <c r="F49">
-        <v>6.922087066782793E-05</v>
+        <v>0.7218993854749942</v>
       </c>
       <c r="G49">
-        <v>0.003630510390706761</v>
+        <v>0.008815401466899679</v>
       </c>
       <c r="H49">
         <v>132</v>
       </c>
       <c r="I49">
-        <v>1.211209706726751</v>
+        <v>0.4716679386076486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Summer Calculation error
</commit_message>
<xml_diff>
--- a/output/palmer_drought_trendlines/region/Decade.xlsx
+++ b/output/palmer_drought_trendlines/region/Decade.xlsx
@@ -73,12 +73,12 @@
     <t>Spring Wheat Belt (area weighted)</t>
   </si>
   <si>
+    <t>Cotton Belt (area weighted)</t>
+  </si>
+  <si>
     <t>West North Central Region</t>
   </si>
   <si>
-    <t>Cotton Belt (area weighted)</t>
-  </si>
-  <si>
     <t>Missouri River Basin</t>
   </si>
   <si>
@@ -88,18 +88,18 @@
     <t>Pacific Northwest Basin</t>
   </si>
   <si>
+    <t>Cotton Belt (productivity weighted)</t>
+  </si>
+  <si>
     <t>Northwest Region</t>
   </si>
   <si>
-    <t>Cotton Belt (productivity weighted)</t>
+    <t>Contiguous 48 States</t>
   </si>
   <si>
     <t>Southeast Region</t>
   </si>
   <si>
-    <t>Contiguous 48 States</t>
-  </si>
-  <si>
     <t>South Atlantic-Gulf Basin</t>
   </si>
   <si>
@@ -115,10 +115,10 @@
     <t>Spring Wheat Belt (productivity weighted)</t>
   </si>
   <si>
+    <t>Southern Plains and Gulf Coast</t>
+  </si>
+  <si>
     <t>NWS Eastern Region</t>
-  </si>
-  <si>
-    <t>Southern Plains and Gulf Coast</t>
   </si>
   <si>
     <t>Arkansas-White-Red Basin</t>
@@ -582,25 +582,25 @@
         <v>9</v>
       </c>
       <c r="C2">
-        <v>-0.04139514314228129</v>
+        <v>-0.03139849258686706</v>
       </c>
       <c r="D2">
-        <v>2.271755278555077</v>
+        <v>1.841130331552617</v>
       </c>
       <c r="E2">
-        <v>-0.337080597389853</v>
+        <v>-0.3610638894924244</v>
       </c>
       <c r="F2">
-        <v>7.742542704136124E-05</v>
+        <v>2.107001854344476E-05</v>
       </c>
       <c r="G2">
-        <v>0.01014035399186529</v>
+        <v>0.007112479684085199</v>
       </c>
       <c r="H2">
         <v>132</v>
       </c>
       <c r="I2">
-        <v>-3.109613329941491</v>
+        <v>-2.240673704740101</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -611,25 +611,25 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <v>-0.03617100626838608</v>
+        <v>-0.02616774161986577</v>
       </c>
       <c r="D3">
-        <v>1.800273721699314</v>
+        <v>1.369363859916901</v>
       </c>
       <c r="E3">
-        <v>-0.3017307461159452</v>
+        <v>-0.3149708538860098</v>
       </c>
       <c r="F3">
-        <v>0.0004381622399571161</v>
+        <v>0.0002347003961840106</v>
       </c>
       <c r="G3">
-        <v>0.01002400764620268</v>
+        <v>0.006915710220606137</v>
       </c>
       <c r="H3">
         <v>132</v>
       </c>
       <c r="I3">
-        <v>-2.901957093190877</v>
+        <v>-2.03244255066565</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -640,25 +640,25 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>-0.03531165293622686</v>
+        <v>-0.02502673815627264</v>
       </c>
       <c r="D4">
-        <v>1.726928008140424</v>
+        <v>1.283885525311626</v>
       </c>
       <c r="E4">
-        <v>-0.3105972414292575</v>
+        <v>-0.3248602812568758</v>
       </c>
       <c r="F4">
-        <v>0.0002893863740246028</v>
+        <v>0.0001444212126258749</v>
       </c>
       <c r="G4">
-        <v>0.009478069962919222</v>
+        <v>0.006390249677286304</v>
       </c>
       <c r="H4">
         <v>132</v>
       </c>
       <c r="I4">
-        <v>-2.863586873569068</v>
+        <v>-1.969590435003817</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -669,25 +669,25 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>-0.03474710421436446</v>
+        <v>-0.02416014584923261</v>
       </c>
       <c r="D5">
-        <v>1.683413720003393</v>
+        <v>1.22736012889002</v>
       </c>
       <c r="E5">
-        <v>-0.3127304884033399</v>
+        <v>-0.3143875426548785</v>
       </c>
       <c r="F5">
-        <v>0.00026138726828553</v>
+        <v>0.0002413940815933129</v>
       </c>
       <c r="G5">
-        <v>0.009256100100688424</v>
+        <v>0.006398285478898368</v>
       </c>
       <c r="H5">
         <v>132</v>
       </c>
       <c r="I5">
-        <v>-2.833709827863988</v>
+        <v>-1.913458831510219</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -698,25 +698,25 @@
         <v>13</v>
       </c>
       <c r="C6">
-        <v>-0.03227526890136914</v>
+        <v>-0.02219043043787385</v>
       </c>
       <c r="D6">
-        <v>1.569325192911049</v>
+        <v>1.134901382175868</v>
       </c>
       <c r="E6">
-        <v>-0.2636952356758397</v>
+        <v>-0.2539225453768214</v>
       </c>
       <c r="F6">
-        <v>0.002250044569678197</v>
+        <v>0.003304323020392192</v>
       </c>
       <c r="G6">
-        <v>0.01035489952601771</v>
+        <v>0.007413445534272188</v>
       </c>
       <c r="H6">
         <v>132</v>
       </c>
       <c r="I6">
-        <v>-2.626459764266939</v>
+        <v>-1.749854574747733</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -727,25 +727,25 @@
         <v>14</v>
       </c>
       <c r="C7">
-        <v>-0.03139422604021944</v>
+        <v>-0.02073230795321868</v>
       </c>
       <c r="D7">
-        <v>1.547124056643772</v>
+        <v>1.087841431357586</v>
       </c>
       <c r="E7">
-        <v>-0.2999561636476684</v>
+        <v>-0.3047101750848071</v>
       </c>
       <c r="F7">
-        <v>0.0004753526501403797</v>
+        <v>0.0003817042199122878</v>
       </c>
       <c r="G7">
-        <v>0.008756837409324552</v>
+        <v>0.005683671642042947</v>
       </c>
       <c r="H7">
         <v>132</v>
       </c>
       <c r="I7">
-        <v>-2.534125328584754</v>
+        <v>-1.607358602560842</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -756,25 +756,25 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>-0.02858190451963031</v>
+        <v>-0.01824462816925295</v>
       </c>
       <c r="D8">
-        <v>1.321528194691767</v>
+        <v>0.8762301365216659</v>
       </c>
       <c r="E8">
-        <v>-0.261836986551212</v>
+        <v>-0.2578914224123673</v>
       </c>
       <c r="F8">
-        <v>0.002423288308762381</v>
+        <v>0.002831747888339994</v>
       </c>
       <c r="G8">
-        <v>0.00923987850449612</v>
+        <v>0.00599489728715521</v>
       </c>
       <c r="H8">
         <v>132</v>
       </c>
       <c r="I8">
-        <v>-2.394119392860172</v>
+        <v>-1.495571525481218</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -785,25 +785,25 @@
         <v>16</v>
       </c>
       <c r="C9">
-        <v>-0.02856707042639376</v>
+        <v>-0.01811404744666002</v>
       </c>
       <c r="D9">
-        <v>1.272948359196134</v>
+        <v>0.8226642923768345</v>
       </c>
       <c r="E9">
-        <v>-0.2434649843393746</v>
+        <v>-0.2152733213536898</v>
       </c>
       <c r="F9">
-        <v>0.004907362549638044</v>
+        <v>0.01317828612517916</v>
       </c>
       <c r="G9">
-        <v>0.009981339263671994</v>
+        <v>0.007206921710432555</v>
       </c>
       <c r="H9">
         <v>132</v>
       </c>
       <c r="I9">
-        <v>-2.440770796235055</v>
+        <v>-1.532161875688969</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -814,25 +814,25 @@
         <v>17</v>
       </c>
       <c r="C10">
-        <v>-0.02628635109484768</v>
+        <v>-0.01581899758005076</v>
       </c>
       <c r="D10">
-        <v>1.274122106334267</v>
+        <v>0.8232207241583998</v>
       </c>
       <c r="E10">
-        <v>-0.2457887378624516</v>
+        <v>-0.2300855495475199</v>
       </c>
       <c r="F10">
-        <v>0.004500727095305147</v>
+        <v>0.007953300357696338</v>
       </c>
       <c r="G10">
-        <v>0.009092124112793688</v>
+        <v>0.00586822602977849</v>
       </c>
       <c r="H10">
         <v>132</v>
       </c>
       <c r="I10">
-        <v>-2.143103535995931</v>
+        <v>-1.233248961248199</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -843,83 +843,83 @@
         <v>18</v>
       </c>
       <c r="C11">
-        <v>-0.02272196283323224</v>
+        <v>-0.01219949187588465</v>
       </c>
       <c r="D11">
-        <v>1.67842143644535</v>
+        <v>1.22514576443653</v>
       </c>
       <c r="E11">
-        <v>-0.1936126638574839</v>
+        <v>-0.1463001527423867</v>
       </c>
       <c r="F11">
-        <v>0.02612324494640033</v>
+        <v>0.09415164785988391</v>
       </c>
       <c r="G11">
-        <v>0.01009819997947849</v>
+        <v>0.007234808887941559</v>
       </c>
       <c r="H11">
         <v>132</v>
       </c>
       <c r="I11">
-        <v>-1.275433731874842</v>
+        <v>-0.3607881794284744</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
         <v>19</v>
       </c>
       <c r="C12">
-        <v>-0.02211913455831034</v>
+        <v>-0.01164267720746989</v>
       </c>
       <c r="D12">
-        <v>1.803972186890528</v>
+        <v>0.6635938268464346</v>
       </c>
       <c r="E12">
-        <v>-0.1843308831938877</v>
+        <v>-0.1520048111112486</v>
       </c>
       <c r="F12">
-        <v>0.034359819571199</v>
+        <v>0.0818735411642484</v>
       </c>
       <c r="G12">
-        <v>0.01034408039449808</v>
+        <v>0.006639688228224658</v>
       </c>
       <c r="H12">
         <v>132</v>
       </c>
       <c r="I12">
-        <v>-1.071515305689816</v>
+        <v>-0.8499542101246506</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13">
-        <v>-0.02164318598386267</v>
+        <v>-0.01157737249607004</v>
       </c>
       <c r="D13">
-        <v>1.094384974137201</v>
+        <v>1.349865513440177</v>
       </c>
       <c r="E13">
-        <v>-0.186838774898026</v>
+        <v>-0.1331458616700852</v>
       </c>
       <c r="F13">
-        <v>0.03194290485987202</v>
+        <v>0.1280179350578363</v>
       </c>
       <c r="G13">
-        <v>0.009980830917127408</v>
+        <v>0.007558342712078736</v>
       </c>
       <c r="H13">
         <v>132</v>
       </c>
       <c r="I13">
-        <v>-1.719229203764946</v>
+        <v>-0.1551929110489279</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -930,25 +930,25 @@
         <v>21</v>
       </c>
       <c r="C14">
-        <v>-0.01892619480917624</v>
+        <v>-0.008456636596677305</v>
       </c>
       <c r="D14">
-        <v>1.635104723140847</v>
+        <v>1.184108369371662</v>
       </c>
       <c r="E14">
-        <v>-0.1554692001344543</v>
+        <v>-0.09553217064559839</v>
       </c>
       <c r="F14">
-        <v>0.0750667777709185</v>
+        <v>0.2758734960074624</v>
       </c>
       <c r="G14">
-        <v>0.01054712756796859</v>
+        <v>0.007728326759848208</v>
       </c>
       <c r="H14">
         <v>132</v>
       </c>
       <c r="I14">
-        <v>-0.8253006020520652</v>
+        <v>0.08474561180361206</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -959,25 +959,25 @@
         <v>22</v>
       </c>
       <c r="C15">
-        <v>-0.018739319935555</v>
+        <v>-0.008275824641736634</v>
       </c>
       <c r="D15">
-        <v>1.636309166454677</v>
+        <v>1.185573984567117</v>
       </c>
       <c r="E15">
-        <v>-0.1561498088603786</v>
+        <v>-0.09618433490405821</v>
       </c>
       <c r="F15">
-        <v>0.07378478231576593</v>
+        <v>0.2725936635951405</v>
       </c>
       <c r="G15">
-        <v>0.01039633882955093</v>
+        <v>0.007511332467556107</v>
       </c>
       <c r="H15">
         <v>132</v>
       </c>
       <c r="I15">
-        <v>-0.7998024251674727</v>
+        <v>0.1097167811413544</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -988,141 +988,141 @@
         <v>23</v>
       </c>
       <c r="C16">
-        <v>-0.01715543771076716</v>
+        <v>-0.006539818275508943</v>
       </c>
       <c r="D16">
-        <v>0.6193979479352166</v>
+        <v>0.1621097261087088</v>
       </c>
       <c r="E16">
-        <v>-0.1781867399206297</v>
+        <v>-0.1224558830024464</v>
       </c>
       <c r="F16">
-        <v>0.04094099022317375</v>
+        <v>0.161873001539701</v>
       </c>
       <c r="G16">
-        <v>0.008308992797725694</v>
+        <v>0.004648720869822602</v>
       </c>
       <c r="H16">
         <v>132</v>
       </c>
       <c r="I16">
-        <v>-1.610808954464514</v>
+        <v>-0.6880666497074537</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
       </c>
       <c r="C17">
-        <v>-0.01631631671982728</v>
+        <v>-0.00584422506180329</v>
       </c>
       <c r="D17">
-        <v>0.555846858305775</v>
+        <v>0.2732186890528282</v>
       </c>
       <c r="E17">
-        <v>-0.1692474081945817</v>
+        <v>-0.08810444798780348</v>
       </c>
       <c r="F17">
-        <v>0.05237607573357037</v>
+        <v>0.3151037183116861</v>
       </c>
       <c r="G17">
-        <v>0.008333308973065154</v>
+        <v>0.005795157760149652</v>
       </c>
       <c r="H17">
         <v>132</v>
       </c>
       <c r="I17">
-        <v>-1.565274315271772</v>
+        <v>-0.4865305689815994</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
       </c>
       <c r="C18">
-        <v>-0.01594229171151074</v>
+        <v>-0.005729909529120929</v>
       </c>
       <c r="D18">
-        <v>0.7082123293479186</v>
+        <v>0.09981701009073202</v>
       </c>
       <c r="E18">
-        <v>-0.146821513765262</v>
+        <v>-0.1078219875983904</v>
       </c>
       <c r="F18">
-        <v>0.09297220942991884</v>
+        <v>0.2184766076233898</v>
       </c>
       <c r="G18">
-        <v>0.009420137491761094</v>
+        <v>0.004633716972627595</v>
       </c>
       <c r="H18">
         <v>132</v>
       </c>
       <c r="I18">
-        <v>-1.364285593148478</v>
+        <v>-0.6450712286949887</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
       </c>
       <c r="C19">
-        <v>-0.01426078964705269</v>
+        <v>-0.003778846643054227</v>
       </c>
       <c r="D19">
-        <v>0.5930920037310273</v>
+        <v>0.4032860171288054</v>
       </c>
       <c r="E19">
-        <v>-0.1476641176195292</v>
+        <v>-0.05549586688397131</v>
       </c>
       <c r="F19">
-        <v>0.09109085780724646</v>
+        <v>0.5273725243805378</v>
       </c>
       <c r="G19">
-        <v>0.008377408844499806</v>
+        <v>0.005962894852972175</v>
       </c>
       <c r="H19">
         <v>132</v>
       </c>
       <c r="I19">
-        <v>-1.260810650385823</v>
+        <v>-0.08796404646824407</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
       </c>
       <c r="C20">
-        <v>-0.01415194933108951</v>
+        <v>-0.003625879106901749</v>
       </c>
       <c r="D20">
-        <v>0.8501273636903252</v>
+        <v>0.1349727804629866</v>
       </c>
       <c r="E20">
-        <v>-0.1311743862188633</v>
+        <v>-0.06742841805502356</v>
       </c>
       <c r="F20">
-        <v>0.1338137762503171</v>
+        <v>0.442368303506281</v>
       </c>
       <c r="G20">
-        <v>0.009380514028818012</v>
+        <v>0.004705536450353868</v>
       </c>
       <c r="H20">
         <v>132</v>
       </c>
       <c r="I20">
-        <v>-0.9896260493513106</v>
+        <v>-0.3363915034342407</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1133,25 +1133,25 @@
         <v>28</v>
       </c>
       <c r="C21">
-        <v>-0.01400653973347945</v>
+        <v>-0.003328637588138989</v>
       </c>
       <c r="D21">
-        <v>0.584143644534894</v>
+        <v>0.124172475197151</v>
       </c>
       <c r="E21">
-        <v>-0.1454239875277568</v>
+        <v>-0.06158900199116489</v>
       </c>
       <c r="F21">
-        <v>0.09616040879051212</v>
+        <v>0.4829660900719859</v>
       </c>
       <c r="G21">
-        <v>0.008357600711645338</v>
+        <v>0.004731146759728398</v>
       </c>
       <c r="H21">
         <v>132</v>
       </c>
       <c r="I21">
-        <v>-1.236706520817434</v>
+        <v>-0.3085504112609175</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1162,25 +1162,25 @@
         <v>29</v>
       </c>
       <c r="C22">
-        <v>-0.01346308174992989</v>
+        <v>-0.002908642675902917</v>
       </c>
       <c r="D22">
-        <v>0.9373998134486564</v>
+        <v>0.4827470533367253</v>
       </c>
       <c r="E22">
-        <v>-0.1202424119937283</v>
+        <v>-0.03813109067947308</v>
       </c>
       <c r="F22">
-        <v>0.1696501584111955</v>
+        <v>0.664227434098662</v>
       </c>
       <c r="G22">
-        <v>0.009748833283525426</v>
+        <v>0.006685340170942798</v>
       </c>
       <c r="H22">
         <v>132</v>
       </c>
       <c r="I22">
-        <v>-0.812800814042229</v>
+        <v>0.1046235054693461</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1191,25 +1191,25 @@
         <v>30</v>
       </c>
       <c r="C23">
-        <v>-0.01171556920989636</v>
+        <v>-0.0008877476208180887</v>
       </c>
       <c r="D23">
-        <v>1.330146018824727</v>
+        <v>0.8637167811413552</v>
       </c>
       <c r="E23">
-        <v>-0.1101117420293871</v>
+        <v>-0.01261182327812399</v>
       </c>
       <c r="F23">
-        <v>0.2087967948026354</v>
+        <v>0.8858744970199526</v>
       </c>
       <c r="G23">
-        <v>0.009274898608498446</v>
+        <v>0.00617312999495848</v>
       </c>
       <c r="H23">
         <v>132</v>
       </c>
       <c r="I23">
-        <v>-0.1928779784617998</v>
+        <v>0.7483095904350037</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1220,25 +1220,25 @@
         <v>31</v>
       </c>
       <c r="C24">
-        <v>-0.01112215590735052</v>
+        <v>-0.00083999699952384</v>
       </c>
       <c r="D24">
-        <v>0.3884139743915886</v>
+        <v>-0.05450979394556081</v>
       </c>
       <c r="E24">
-        <v>-0.1008370005386396</v>
+        <v>-0.01177643212151656</v>
       </c>
       <c r="F24">
-        <v>0.2499606696417918</v>
+        <v>0.8933878110398364</v>
       </c>
       <c r="G24">
-        <v>0.009624498440692549</v>
+        <v>0.00625550259248005</v>
       </c>
       <c r="H24">
         <v>132</v>
       </c>
       <c r="I24">
-        <v>-1.057466293563979</v>
+        <v>-0.16370940388366</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1249,83 +1249,83 @@
         <v>32</v>
       </c>
       <c r="C25">
-        <v>-0.01109717237735555</v>
+        <v>-0.0002941536374250672</v>
       </c>
       <c r="D25">
-        <v>1.208154328839143</v>
+        <v>0.7427935215805985</v>
       </c>
       <c r="E25">
-        <v>-0.09765996738072406</v>
+        <v>-0.003641485495796595</v>
       </c>
       <c r="F25">
-        <v>0.26527014925123</v>
+        <v>0.966945369636388</v>
       </c>
       <c r="G25">
-        <v>0.009918433972281317</v>
+        <v>0.007084693770659145</v>
       </c>
       <c r="H25">
         <v>132</v>
       </c>
       <c r="I25">
-        <v>-0.2344780802170787</v>
+        <v>0.7045535487153398</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
         <v>33</v>
       </c>
       <c r="C26">
-        <v>-0.01060097319792054</v>
+        <v>-0.0002512833558369029</v>
       </c>
       <c r="D26">
-        <v>0.6505389637920803</v>
+        <v>-0.1941261765454084</v>
       </c>
       <c r="E26">
-        <v>-0.1127092630420259</v>
+        <v>-0.003285547432852824</v>
       </c>
       <c r="F26">
-        <v>0.1981923509912407</v>
+        <v>0.9701747356941263</v>
       </c>
       <c r="G26">
-        <v>0.008196685573309574</v>
+        <v>0.006707828674526767</v>
       </c>
       <c r="H26">
         <v>132</v>
       </c>
       <c r="I26">
-        <v>-0.7275875519375904</v>
+        <v>-0.2267930128042058</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
         <v>34</v>
       </c>
       <c r="C27">
-        <v>-0.01059903202029888</v>
+        <v>6.149606350573025E-05</v>
       </c>
       <c r="D27">
-        <v>0.2516229966929538</v>
+        <v>0.1912325956075638</v>
       </c>
       <c r="E27">
-        <v>-0.09375859925324567</v>
+        <v>0.001264732617639735</v>
       </c>
       <c r="F27">
-        <v>0.2849271762118099</v>
+        <v>0.9885168651777769</v>
       </c>
       <c r="G27">
-        <v>0.009871112628624003</v>
+        <v>0.004264583024500008</v>
       </c>
       <c r="H27">
         <v>132</v>
       </c>
       <c r="I27">
-        <v>-1.1262511659459</v>
+        <v>0.1992270838633088</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1336,25 +1336,25 @@
         <v>35</v>
       </c>
       <c r="C28">
-        <v>-0.009172651312056046</v>
+        <v>0.001328323842696776</v>
       </c>
       <c r="D28">
-        <v>0.6411650979394559</v>
+        <v>0.188815398965488</v>
       </c>
       <c r="E28">
-        <v>-0.08459230737400661</v>
+        <v>0.0188875645754022</v>
       </c>
       <c r="F28">
-        <v>0.3348566203071313</v>
+        <v>0.8298009844261096</v>
       </c>
       <c r="G28">
-        <v>0.00947617071676689</v>
+        <v>0.006167069614166169</v>
       </c>
       <c r="H28">
         <v>132</v>
       </c>
       <c r="I28">
-        <v>-0.5512795726278301</v>
+        <v>0.3614974985160689</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1365,25 +1365,25 @@
         <v>36</v>
       </c>
       <c r="C29">
-        <v>-0.008541154139678694</v>
+        <v>0.002177534913149262</v>
       </c>
       <c r="D29">
-        <v>0.4129049436106169</v>
+        <v>-0.04882320020351064</v>
       </c>
       <c r="E29">
-        <v>-0.09128456698547943</v>
+        <v>0.04431609158129247</v>
       </c>
       <c r="F29">
-        <v>0.2978848877178756</v>
+        <v>0.6138689898341607</v>
       </c>
       <c r="G29">
-        <v>0.008172039971839774</v>
+        <v>0.004305316874228761</v>
       </c>
       <c r="H29">
         <v>132</v>
       </c>
       <c r="I29">
-        <v>-0.6974450945476134</v>
+        <v>0.2342563385058934</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1394,25 +1394,25 @@
         <v>37</v>
       </c>
       <c r="C30">
-        <v>-0.0076459933859069</v>
+        <v>0.002823564826592049</v>
       </c>
       <c r="D30">
-        <v>0.616186381751887</v>
+        <v>0.1651900279827013</v>
       </c>
       <c r="E30">
-        <v>-0.07027766620948486</v>
+        <v>0.04016093255000773</v>
       </c>
       <c r="F30">
-        <v>0.423282178048217</v>
+        <v>0.6475201720226642</v>
       </c>
       <c r="G30">
-        <v>0.009518527615568142</v>
+        <v>0.006161291816218183</v>
       </c>
       <c r="H30">
         <v>132</v>
       </c>
       <c r="I30">
-        <v>-0.37779275841601</v>
+        <v>0.5322534554396677</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1423,25 +1423,25 @@
         <v>38</v>
       </c>
       <c r="C31">
-        <v>-0.007337770124389307</v>
+        <v>0.003179740263128718</v>
       </c>
       <c r="D31">
-        <v>0.6308735690663954</v>
+        <v>0.1778115831425419</v>
       </c>
       <c r="E31">
-        <v>-0.06669628438731372</v>
+        <v>0.04373513832364177</v>
       </c>
       <c r="F31">
-        <v>0.4473500435800749</v>
+        <v>0.6185279756851472</v>
       </c>
       <c r="G31">
-        <v>0.009627702774319669</v>
+        <v>0.006370502885075133</v>
       </c>
       <c r="H31">
         <v>132</v>
       </c>
       <c r="I31">
-        <v>-0.3230365471042145</v>
+        <v>0.5911778173492752</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1452,25 +1452,25 @@
         <v>39</v>
       </c>
       <c r="C32">
-        <v>-0.006346183198638048</v>
+        <v>0.004080934583096885</v>
       </c>
       <c r="D32">
-        <v>0.1371610277283136</v>
+        <v>-0.3120071228694991</v>
       </c>
       <c r="E32">
-        <v>-0.0570861314870384</v>
+        <v>0.05494571473060438</v>
       </c>
       <c r="F32">
-        <v>0.5155875207511315</v>
+        <v>0.5314809330937141</v>
       </c>
       <c r="G32">
-        <v>0.009734228006570016</v>
+        <v>0.00650425506739873</v>
       </c>
       <c r="H32">
         <v>132</v>
       </c>
       <c r="I32">
-        <v>-0.6878427880946327</v>
+        <v>0.2185143729330961</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1481,25 +1481,25 @@
         <v>40</v>
       </c>
       <c r="C33">
-        <v>-0.005375110397954461</v>
+        <v>0.005400349620700679</v>
       </c>
       <c r="D33">
-        <v>0.2093223098448234</v>
+        <v>-0.2548513524972443</v>
       </c>
       <c r="E33">
-        <v>-0.05791762994862039</v>
+        <v>0.1106589548969623</v>
       </c>
       <c r="F33">
-        <v>0.5094797590737756</v>
+        <v>0.206529673143357</v>
       </c>
       <c r="G33">
-        <v>0.008125971526367329</v>
+        <v>0.004253908715959724</v>
       </c>
       <c r="H33">
         <v>132</v>
       </c>
       <c r="I33">
-        <v>-0.4894420418892564</v>
+        <v>0.447194098193844</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1510,25 +1510,25 @@
         <v>41</v>
       </c>
       <c r="C34">
-        <v>-0.004730454180772167</v>
+        <v>0.005786505032320349</v>
       </c>
       <c r="D34">
-        <v>-0.1428616976172304</v>
+        <v>-0.5958999406427543</v>
       </c>
       <c r="E34">
-        <v>-0.04243563364357255</v>
+        <v>0.07594705262882763</v>
       </c>
       <c r="F34">
-        <v>0.6290042408869247</v>
+        <v>0.3867551038511022</v>
       </c>
       <c r="G34">
-        <v>0.009768077241313478</v>
+        <v>0.006663119666809093</v>
       </c>
       <c r="H34">
         <v>132</v>
       </c>
       <c r="I34">
-        <v>-0.7578207411176121</v>
+        <v>0.156345713558891</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1539,25 +1539,25 @@
         <v>42</v>
       </c>
       <c r="C35">
-        <v>-0.004600700545956208</v>
+        <v>0.006169247728443864</v>
       </c>
       <c r="D35">
-        <v>0.5269098617824135</v>
+        <v>0.06297362842364101</v>
       </c>
       <c r="E35">
-        <v>-0.04453821376355798</v>
+        <v>0.0940341559429983</v>
       </c>
       <c r="F35">
-        <v>0.6120917194266923</v>
+        <v>0.2835076389527921</v>
       </c>
       <c r="G35">
-        <v>0.009050828224642864</v>
+        <v>0.005728570415692607</v>
       </c>
       <c r="H35">
         <v>132</v>
       </c>
       <c r="I35">
-        <v>-0.07118120919189352</v>
+        <v>0.8649758331213433</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1568,25 +1568,25 @@
         <v>43</v>
       </c>
       <c r="C36">
-        <v>-0.003576915901871386</v>
+        <v>0.00722389814035706</v>
       </c>
       <c r="D36">
-        <v>0.5506939709997458</v>
+        <v>0.08542813533452015</v>
       </c>
       <c r="E36">
-        <v>-0.03426917256478689</v>
+        <v>0.1070014442798854</v>
       </c>
       <c r="F36">
-        <v>0.6964680347123431</v>
+        <v>0.2220217832881242</v>
       </c>
       <c r="G36">
-        <v>0.009149097850015055</v>
+        <v>0.005887213282334463</v>
       </c>
       <c r="H36">
         <v>132</v>
       </c>
       <c r="I36">
-        <v>0.0856949037564656</v>
+        <v>1.024534893580938</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1597,25 +1597,25 @@
         <v>44</v>
       </c>
       <c r="C37">
-        <v>-0.002987117520823957</v>
+        <v>0.007792200718809728</v>
       </c>
       <c r="D37">
-        <v>0.06932671924022732</v>
+        <v>-0.3950131433901469</v>
       </c>
       <c r="E37">
-        <v>-0.03260421133510322</v>
+        <v>0.1675039297723741</v>
       </c>
       <c r="F37">
-        <v>0.7105409087704093</v>
+        <v>0.0548887303006447</v>
       </c>
       <c r="G37">
-        <v>0.008031117422189357</v>
+        <v>0.00402238582952408</v>
       </c>
       <c r="H37">
         <v>132</v>
       </c>
       <c r="I37">
-        <v>-0.3189985584668871</v>
+        <v>0.6179729500551177</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1626,25 +1626,25 @@
         <v>45</v>
       </c>
       <c r="C38">
-        <v>-0.002830833153957043</v>
+        <v>0.007903839957210607</v>
       </c>
       <c r="D38">
-        <v>-0.1248493173916729</v>
+        <v>-0.5872660052573565</v>
       </c>
       <c r="E38">
-        <v>-0.02947643138667949</v>
+        <v>0.1450825431038305</v>
       </c>
       <c r="F38">
-        <v>0.7372401883157859</v>
+        <v>0.09695234894293332</v>
       </c>
       <c r="G38">
-        <v>0.008419357306524928</v>
+        <v>0.004727502765268557</v>
       </c>
       <c r="H38">
         <v>132</v>
       </c>
       <c r="I38">
-        <v>-0.4928576274060885</v>
+        <v>0.4402331891800223</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1655,25 +1655,25 @@
         <v>46</v>
       </c>
       <c r="C39">
-        <v>-0.002061627171268483</v>
+        <v>0.008767847941086307</v>
       </c>
       <c r="D39">
-        <v>0.1927533282455694</v>
+        <v>-0.2737471381327909</v>
       </c>
       <c r="E39">
-        <v>-0.02174111917405279</v>
+        <v>0.1657269671420314</v>
       </c>
       <c r="F39">
-        <v>0.8045677845257424</v>
+        <v>0.05755103158689211</v>
       </c>
       <c r="G39">
-        <v>0.008314839910834574</v>
+        <v>0.00457594372563546</v>
       </c>
       <c r="H39">
         <v>132</v>
       </c>
       <c r="I39">
-        <v>-0.07525820401933342</v>
+        <v>0.8660730942084289</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1684,25 +1684,25 @@
         <v>47</v>
       </c>
       <c r="C40">
-        <v>0.0007342086896398799</v>
+        <v>0.01158187255803639</v>
       </c>
       <c r="D40">
-        <v>0.1826644619689645</v>
+        <v>-0.28461952005427</v>
       </c>
       <c r="E40">
-        <v>0.007316953672887244</v>
+        <v>0.1865905427078574</v>
       </c>
       <c r="F40">
-        <v>0.9336392840289326</v>
+        <v>0.03217552498662146</v>
       </c>
       <c r="G40">
-        <v>0.008800470933456725</v>
+        <v>0.005348383346911447</v>
       </c>
       <c r="H40">
         <v>132</v>
       </c>
       <c r="I40">
-        <v>0.2781115916221488</v>
+        <v>1.221023912490461</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -1713,25 +1713,25 @@
         <v>48</v>
       </c>
       <c r="C41">
-        <v>0.001042752871651372</v>
+        <v>0.01192569190328032</v>
       </c>
       <c r="D41">
-        <v>-0.1316089205460867</v>
+        <v>-0.6004124480624107</v>
       </c>
       <c r="E41">
-        <v>0.01081327883063006</v>
+        <v>0.2090777976995488</v>
       </c>
       <c r="F41">
-        <v>0.9020618974316522</v>
+        <v>0.01613148370161881</v>
       </c>
       <c r="G41">
-        <v>0.008457206300937121</v>
+        <v>0.004892130109929857</v>
       </c>
       <c r="H41">
         <v>132</v>
       </c>
       <c r="I41">
-        <v>0.003948952768591613</v>
+        <v>0.9499274993640303</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -1742,25 +1742,25 @@
         <v>49</v>
       </c>
       <c r="C42">
-        <v>0.001146141452882744</v>
+        <v>0.01207537913625424</v>
       </c>
       <c r="D42">
-        <v>-0.1218653438480456</v>
+        <v>-0.5926632748240486</v>
       </c>
       <c r="E42">
-        <v>0.01221387317811288</v>
+        <v>0.2262711222959392</v>
       </c>
       <c r="F42">
-        <v>0.8894523451003896</v>
+        <v>0.009084485658546379</v>
       </c>
       <c r="G42">
-        <v>0.008229638177953332</v>
+        <v>0.004559189270953317</v>
       </c>
       <c r="H42">
         <v>132</v>
       </c>
       <c r="I42">
-        <v>0.02713304502671107</v>
+        <v>0.9771360128890025</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1771,25 +1771,25 @@
         <v>50</v>
       </c>
       <c r="C43">
-        <v>0.001529041347866078</v>
+        <v>0.01239709867000633</v>
       </c>
       <c r="D43">
-        <v>0.06554583227338232</v>
+        <v>-0.4026166369880442</v>
       </c>
       <c r="E43">
-        <v>0.01529137428838767</v>
+        <v>0.199919827904557</v>
       </c>
       <c r="F43">
-        <v>0.8618468272478064</v>
+        <v>0.02154411325198093</v>
       </c>
       <c r="G43">
-        <v>0.008769003716384246</v>
+        <v>0.005328873136014267</v>
       </c>
       <c r="H43">
         <v>132</v>
       </c>
       <c r="I43">
-        <v>0.2643212074959725</v>
+        <v>1.209006190112779</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -1800,25 +1800,25 @@
         <v>51</v>
       </c>
       <c r="C44">
-        <v>0.001534016920076445</v>
+        <v>0.01254537959284843</v>
       </c>
       <c r="D44">
-        <v>0.06678317646061233</v>
+        <v>-0.4075524463664889</v>
       </c>
       <c r="E44">
-        <v>0.01608230861241003</v>
+        <v>0.2205578901861404</v>
       </c>
       <c r="F44">
-        <v>0.8547775491175317</v>
+        <v>0.01104437244546879</v>
       </c>
       <c r="G44">
-        <v>0.008364768220067193</v>
+        <v>0.004865871721311882</v>
       </c>
       <c r="H44">
         <v>132</v>
       </c>
       <c r="I44">
-        <v>0.2662053760705502</v>
+        <v>1.223346900703807</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -1829,25 +1829,25 @@
         <v>52</v>
       </c>
       <c r="C45">
-        <v>0.001811862317280784</v>
+        <v>0.01283424847856291</v>
       </c>
       <c r="D45">
-        <v>0.1399899940642756</v>
+        <v>-0.3348204867294164</v>
       </c>
       <c r="E45">
-        <v>0.01860305976716366</v>
+        <v>0.2134829794191099</v>
       </c>
       <c r="F45">
-        <v>0.8323267761670338</v>
+        <v>0.0139788055535456</v>
       </c>
       <c r="G45">
-        <v>0.008540709952715978</v>
+        <v>0.005151176360905226</v>
       </c>
       <c r="H45">
         <v>132</v>
       </c>
       <c r="I45">
-        <v>0.3755320953107775</v>
+        <v>1.333631815483762</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -1858,25 +1858,25 @@
         <v>53</v>
       </c>
       <c r="C46">
-        <v>0.001958350781754498</v>
+        <v>0.01286223444155269</v>
       </c>
       <c r="D46">
-        <v>0.1050209446281692</v>
+        <v>-0.364684813024676</v>
       </c>
       <c r="E46">
-        <v>0.01928054194778564</v>
+        <v>0.1981851617552829</v>
       </c>
       <c r="F46">
-        <v>0.8263150516329765</v>
+        <v>0.02272886384587612</v>
       </c>
       <c r="G46">
-        <v>0.008906741238857836</v>
+        <v>0.005579208897440417</v>
       </c>
       <c r="H46">
         <v>132</v>
       </c>
       <c r="I46">
-        <v>0.3596065462562539</v>
+        <v>1.307405664377173</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -1887,25 +1887,25 @@
         <v>54</v>
       </c>
       <c r="C47">
-        <v>0.002319669425800183</v>
+        <v>0.0132257577833004</v>
       </c>
       <c r="D47">
-        <v>0.005093530060205131</v>
+        <v>-0.4647071991859582</v>
       </c>
       <c r="E47">
-        <v>0.02346323034333412</v>
+        <v>0.2174378190792962</v>
       </c>
       <c r="F47">
-        <v>0.7894346650380903</v>
+        <v>0.01226420002535472</v>
       </c>
       <c r="G47">
-        <v>0.008668561616183641</v>
+        <v>0.005207108504569252</v>
       </c>
       <c r="H47">
         <v>132</v>
       </c>
       <c r="I47">
-        <v>0.3066505554142289</v>
+        <v>1.254641312643094</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -1916,25 +1916,25 @@
         <v>55</v>
       </c>
       <c r="C48">
-        <v>0.002615143272736762</v>
+        <v>0.01387839265796529</v>
       </c>
       <c r="D48">
-        <v>-0.1466759942338675</v>
+        <v>-0.6318621215975582</v>
       </c>
       <c r="E48">
-        <v>0.02931594946527999</v>
+        <v>0.2681070668256298</v>
       </c>
       <c r="F48">
-        <v>0.7386189008206709</v>
+        <v>0.001882771163329239</v>
       </c>
       <c r="G48">
-        <v>0.007820475224488361</v>
+        <v>0.004373820658256604</v>
       </c>
       <c r="H48">
         <v>132</v>
       </c>
       <c r="I48">
-        <v>0.1932926312219115</v>
+        <v>1.17232892393793</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -1945,25 +1945,25 @@
         <v>56</v>
       </c>
       <c r="C49">
-        <v>0.003144398567598771</v>
+        <v>0.01420646928751737</v>
       </c>
       <c r="D49">
-        <v>0.06289612481980841</v>
+        <v>-0.4136238446536085</v>
       </c>
       <c r="E49">
-        <v>0.03126881341251011</v>
+        <v>0.2161633524251408</v>
       </c>
       <c r="F49">
-        <v>0.7218993854749942</v>
+        <v>0.0127954495174507</v>
       </c>
       <c r="G49">
-        <v>0.008815401466899679</v>
+        <v>0.00562783235611752</v>
       </c>
       <c r="H49">
         <v>132</v>
       </c>
       <c r="I49">
-        <v>0.4716679386076486</v>
+        <v>1.43321716272365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>